<commit_message>
PAUSED (task179): round 1 fix, call frozen at 3,250 with the model form filed by lowest AIC, the continuing-students ask dropped and the teaching-groups ask re-sited to 20 cells on ARC's repeated combination figure against the room; stage 3 green, waiting on a fresh judge and two readers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task179/golden/continuing_enrolment_2027.xlsx
+++ b/task179/golden/continuing_enrolment_2027.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet name="Projection" sheetId="1" r:id="rId1"/>
     <sheet name="Teaching groups S1 2026" sheetId="2" r:id="rId2"/>
-    <sheet name="Continuing 2026 census" sheetId="3" r:id="rId3"/>
-    <sheet name="Notes" sheetId="4" r:id="rId4"/>
+    <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -22,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>Continuing enrolment projection 2027: first-year intake</t>
   </si>
@@ -60,18 +59,27 @@
     <t>Faculty</t>
   </si>
   <si>
-    <t>Teaching groups</t>
-  </si>
-  <si>
-    <t>Over 30 students</t>
-  </si>
-  <si>
-    <t>30 or fewer</t>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>30 students or fewer</t>
+  </si>
+  <si>
+    <t>More than 30</t>
+  </si>
+  <si>
+    <t>Groups</t>
   </si>
   <si>
     <t>Arts and Social Sciences</t>
   </si>
   <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>300 and above</t>
+  </si>
+  <si>
     <t>Business and Law</t>
   </si>
   <si>
@@ -87,15 +95,6 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Year 2</t>
-  </si>
-  <si>
-    <t>Year 3</t>
-  </si>
-  <si>
-    <t>Year 4 or later</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -108,16 +107,13 @@
     <t>Earlier intakes: enrolment at the next census from the census history; the 2025 intake through the SIRIUS to ARC crosswalk.</t>
   </si>
   <si>
-    <t>Projection: logistic model fitted on the 2019 to 2025 intakes (admissions attributes, week-6 progress check, faculty, and the number of other entrants met in two or more Semester 1 classes, banded), applied to the 2026 intake; reported to the nearest 250.</t>
-  </si>
-  <si>
-    <t>Teaching groups: active Semester 1 2026 classes meeting in one room, on one day, at one start, over the same teaching weeks count as one group; size is the census enrolment of its classes.</t>
-  </si>
-  <si>
-    <t>Continuing students: one row per student at the 2026 census; an attempt left enrolled after a transfer approved in ARC is not counted; conjoint students in the first-listed programme's faculty.</t>
-  </si>
-  <si>
-    <t>Sources: Registry census history and first-year cohort extracts; Admissions; Student Success week-6 progress check; Timetabling Semester 1 2026 timetable at the census; Academic Office catalogue; Registry transfers register.</t>
+    <t>Projection: logistic model fitted on the 2019 to 2025 intakes (admissions attributes, week-6 progress check, faculty, and whether the entrant met 10 or more other entrants in two or more Semester 1 classes, the form with the lowest AIC), applied to the 2026 intake; reported to the nearest 250.</t>
+  </si>
+  <si>
+    <t>Teaching groups, 200 level and above: active Semester 1 2026 classes meeting in one room, on one day, at one start, over the same teaching weeks count as one group. Where ARC Scheduling shows the same enrolment on each class of a group, more than the room seats when added, that is the combination's enrolment and is counted once.</t>
+  </si>
+  <si>
+    <t>Sources: Registry census history and first-year cohort extracts; Admissions; Student Success week-6 progress check; Timetabling Semester 1 2026 timetable at the census.</t>
   </si>
 </sst>
 </file>
@@ -533,7 +529,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5">
-        <v>3269.3</v>
+        <v>3253</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -675,16 +671,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0768FF10-B17F-5622-AA27-A86A6F32C7FB}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>11</v>
       </c>
@@ -697,96 +694,204 @@
       <c r="D1" s="6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2">
-        <v>703</v>
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
       </c>
       <c r="C2">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="D2">
-        <f>B2-C2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="E2">
+        <f>C2+D2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3">
-        <v>325</v>
+      <c r="B3" t="s">
+        <v>18</v>
       </c>
       <c r="C3">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="D3">
-        <f>B3-C3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E3">
+        <f>C3+D3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="B4">
-        <v>315</v>
-      </c>
       <c r="C4">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="D4">
-        <f>B4-C4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="E4">
+        <f>C4+D4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5">
-        <v>250</v>
-      </c>
       <c r="C5">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="D5">
-        <f>B5-C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E5">
+        <f>C5+D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6">
-        <v>269</v>
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
       </c>
       <c r="C6">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="D6">
-        <f>B6-C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6">
+        <f>C6+D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3">
-        <f>SUM(B2:B6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="3">
-        <f>SUM(C2:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="3">
-        <f>SUM(D2:D6)</f>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7">
+        <v>18</v>
+      </c>
+      <c r="D7">
+        <v>38</v>
+      </c>
+      <c r="E7">
+        <f>C7+D7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8">
+        <v>15</v>
+      </c>
+      <c r="D8">
+        <v>32</v>
+      </c>
+      <c r="E8">
+        <f>C8+D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9">
+        <v>21</v>
+      </c>
+      <c r="D9">
+        <v>34</v>
+      </c>
+      <c r="E9">
+        <f>C9+D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>13</v>
+      </c>
+      <c r="D10">
+        <v>36</v>
+      </c>
+      <c r="E10">
+        <f>C10+D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11">
+        <v>21</v>
+      </c>
+      <c r="D11">
+        <v>32</v>
+      </c>
+      <c r="E11">
+        <f>C11+D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="3">
+        <f>SUM(C2:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="3">
+        <f>SUM(D2:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="3">
+        <f>SUM(E2:E11)</f>
         <v/>
       </c>
     </row>
@@ -796,149 +901,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B56F01C2-9F7D-5AC6-BC6F-7F36B2E73A02}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1734</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1401</v>
-      </c>
-      <c r="D2" s="2">
-        <v>429</v>
-      </c>
-      <c r="E2" s="2">
-        <f>SUM(B2:D2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1621</v>
-      </c>
-      <c r="C3" s="2">
-        <v>1426</v>
-      </c>
-      <c r="D3" s="2">
-        <v>666</v>
-      </c>
-      <c r="E3" s="2">
-        <f>SUM(B3:D3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1517</v>
-      </c>
-      <c r="C4" s="2">
-        <v>1253</v>
-      </c>
-      <c r="D4" s="2">
-        <v>351</v>
-      </c>
-      <c r="E4" s="2">
-        <f>SUM(B4:D4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="2">
-        <v>1121</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1029</v>
-      </c>
-      <c r="D5" s="2">
-        <v>803</v>
-      </c>
-      <c r="E5" s="2">
-        <f>SUM(B5:D5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="2">
-        <v>1336</v>
-      </c>
-      <c r="C6" s="2">
-        <v>1147</v>
-      </c>
-      <c r="D6" s="2">
-        <v>351</v>
-      </c>
-      <c r="E6" s="2">
-        <f>SUM(B6:D6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="4">
-        <f>SUM(B2:B6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="4">
-        <f>SUM(C2:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
-        <f>SUM(D2:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="4">
-        <f>SUM(E2:E6)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E4F1D2-E066-535A-B29C-44A0B88C07BD}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110.7109375" customWidth="1"/>
@@ -979,11 +943,6 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
PAUSED (task179): rubric repair at stage 4, judge and readers on zip c1b19cef
The portal held the call but both responses answered all 20 S1 2026
teaching-group cells. The asks now stand on two stacked devices: lecture-only
pairs that make three groups, and class lists holding places of students on
leave or with no 2026 census attempt. Call side frozen (freeze.py rubric PASS),
checks 88 green, verify 23, byte-identical rebuilds, ceiling 0 of 20 on all 14
routes. Resume step in task179/pipeline.json.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task179/golden/continuing_enrolment_2027.xlsx
+++ b/task179/golden/continuing_enrolment_2027.xlsx
@@ -110,10 +110,10 @@
     <t>Projection: logistic model fitted on the 2019 to 2025 intakes (admissions attributes, week-6 progress check, faculty, and whether the entrant met 10 or more other entrants in two or more Semester 1 classes, the form with the lowest AIC), applied to the 2026 intake; reported to the nearest 250.</t>
   </si>
   <si>
-    <t>Teaching groups, 200 level and above: active Semester 1 2026 classes meeting in one room, on one day, at one start, over the same teaching weeks count as one group. Where ARC Scheduling shows the same enrolment on each class of a group, more than the room seats when added, that is the combination's enrolment and is counted once.</t>
-  </si>
-  <si>
-    <t>Sources: Registry census history and first-year cohort extracts; Admissions; Student Success week-6 progress check; Timetabling Semester 1 2026 timetable at the census.</t>
+    <t>Teaching groups, 200 level and above: each distinct set of active Semester 1 2026 classes meeting together in one room at one time is a group, so papers sharing only a lecture are the lecture and each workshop. A group's size is the students on its classes' lists who are enrolled at the 2026 census in the census history; places still held by students on approved leave or who left before the census are not counted.</t>
+  </si>
+  <si>
+    <t>Sources: Registry census history and first-year cohort extracts; Admissions; Student Success week-6 progress check; Timetabling Semester 1 2026 timetable at the census; ARC class enrolments at the census.</t>
   </si>
 </sst>
 </file>
@@ -706,10 +706,10 @@
         <v>17</v>
       </c>
       <c r="C2">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E2">
         <f>C2+D2</f>
@@ -724,7 +724,7 @@
         <v>18</v>
       </c>
       <c r="C3">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3">
         <v>45</v>
@@ -742,10 +742,10 @@
         <v>17</v>
       </c>
       <c r="C4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D4">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4">
         <f>C4+D4</f>
@@ -760,10 +760,10 @@
         <v>18</v>
       </c>
       <c r="C5">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D5">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5">
         <f>C5+D5</f>
@@ -778,7 +778,7 @@
         <v>17</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>39</v>
@@ -796,7 +796,7 @@
         <v>18</v>
       </c>
       <c r="C7">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D7">
         <v>38</v>
@@ -814,10 +814,10 @@
         <v>17</v>
       </c>
       <c r="C8">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D8">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E8">
         <f>C8+D8</f>
@@ -832,7 +832,7 @@
         <v>18</v>
       </c>
       <c r="C9">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D9">
         <v>34</v>
@@ -850,7 +850,7 @@
         <v>17</v>
       </c>
       <c r="C10">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D10">
         <v>36</v>
@@ -868,7 +868,7 @@
         <v>18</v>
       </c>
       <c r="C11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D11">
         <v>32</v>

</xml_diff>